<commit_message>
Add release smoke coverage
</commit_message>
<xml_diff>
--- a/registry_template.xlsx
+++ b/registry_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Реестр'!$A$1:$E$1</definedName>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -484,6 +484,31 @@
         <is>
           <t>Сумма долга</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12970001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Тестовый Должник</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>г. Москва, Тестовая улица, д. 1, машиноместо № 0001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>01.01.2026 - 31.01.2026</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1000.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>